<commit_message>
one currency, and it is dollars
The book carried a mix of GBP and USD, from when the rate card quoted both
columns. The practice reads in dollars, and a margin question that answers in
two currencies invites a conversation about exchange rates instead of about
margin.

Fees are re-denominated rather than converted: 485,000 and 560,000 are
fictional round numbers whose job is the gap between them, and putting them
through an exchange rate would turn a clean $75,000 story into $97,000 of
arithmetic nobody asked for. Every relationship the scenes depend on is
therefore untouched.

Per diems and expense thresholds are different and are converted properly,
because those are real local costs rather than a story: a London per diem is
$88 because it was £68. The rate card keeps the USD rates the document had
already authored for itself and drops the GBP column, so there is one number
per level. VAT becomes sales tax.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/sol-internal/trackers-xlsx/Engagements.xlsx
+++ b/demo/sol-internal/trackers-xlsx/Engagements.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">

</xml_diff>